<commit_message>
Avancement des exercices et évolution du modèle de population.
</commit_message>
<xml_diff>
--- a/Maths/Moteur_RTS_evolution_population.xlsx
+++ b/Maths/Moteur_RTS_evolution_population.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trist\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trist\Desktop\moteur_RTS\Maths\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8504301A-82CD-4DAE-B8D2-4ADD0119C001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E1130A-3DD0-4625-B0F9-8108760724B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D398D357-FF3C-4321-AA46-4B35F3AC6ED8}"/>
   </bookViews>
@@ -155,8 +155,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="9.2458223972003498E-2"/>
-          <c:y val="4.6296296296296294E-2"/>
+          <c:x val="0.11190266841644793"/>
+          <c:y val="6.0185185185185182E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -209,12 +209,624 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Feuil1!$B$2:$B$202</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="201"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>53</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>56</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>67</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>69</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>98</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>109</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>123</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>124</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>126</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>127</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>133</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>136</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>139</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>146</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>147</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>149</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>151</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>152</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>154</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>156</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>157</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>158</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>159</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>161</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>162</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>163</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>164</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>166</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>167</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>168</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>169</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>170</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>173</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>176</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>177</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>178</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>179</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>181</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>182</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>183</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>184</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>185</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>186</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>187</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>188</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>189</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>191</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>194</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>196</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>197</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="199">
+                  <c:v>199</c:v>
+                </c:pt>
+                <c:pt idx="200">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$2:$B$102</c:f>
+              <c:f>Feuil1!$B$2:$B$202</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="101"/>
+                <c:ptCount val="201"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -517,6 +1129,306 @@
                 </c:pt>
                 <c:pt idx="100">
                   <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>109</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>123</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>124</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>126</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>127</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>133</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>136</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>139</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>146</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>147</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>149</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>151</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>152</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>154</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>156</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>157</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>158</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>159</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>161</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>162</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>163</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>164</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>166</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>167</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>168</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>169</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>170</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>173</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>176</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>177</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>178</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>179</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>181</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>182</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>183</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>184</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>185</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>186</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>187</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>188</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>189</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>191</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>194</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>196</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>197</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="199">
+                  <c:v>199</c:v>
+                </c:pt>
+                <c:pt idx="200">
+                  <c:v>200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -546,314 +1458,1226 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Feuil1!$B$2:$B$202</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="201"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>53</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>56</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>67</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>69</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>98</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>109</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>123</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>124</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>126</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>127</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>133</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>136</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>139</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>146</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>147</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>149</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>151</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>152</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>154</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>156</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>157</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>158</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>159</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>161</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>162</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>163</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>164</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>166</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>167</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>168</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>169</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>170</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>173</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>176</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>177</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>178</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>179</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>181</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>182</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>183</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>184</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>185</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>186</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>187</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>188</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>189</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>191</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>194</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>196</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>197</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="199">
+                  <c:v>199</c:v>
+                </c:pt>
+                <c:pt idx="200">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$A$2:$A$102</c:f>
+              <c:f>Feuil1!$A$2:$A$202</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="101"/>
+                <c:ptCount val="201"/>
                 <c:pt idx="0">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1025421927520482</c:v>
+                  <c:v>2.0000200001000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2103418361512954</c:v>
+                  <c:v>2.0000400004000025</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.3236684854565661</c:v>
+                  <c:v>2.0000600009000089</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4428055163203397</c:v>
+                  <c:v>2.0000800016000215</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.5680508333754828</c:v>
+                  <c:v>2.0001000025000417</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.6997176151520064</c:v>
+                  <c:v>2.0001200036000721</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.8381350971865147</c:v>
+                  <c:v>2.0001400049001141</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.9836493952825407</c:v>
+                  <c:v>2.0001600064001708</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.1366243709803379</c:v>
+                  <c:v>2.000180008100243</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.2974425414002564</c:v>
+                  <c:v>2.0002000100003334</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.4665060357347905</c:v>
+                  <c:v>2.0002200121004439</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.6442376007810182</c:v>
+                  <c:v>2.0002400144005761</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.8310816580277924</c:v>
+                  <c:v>2.0002600169007323</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.0275054149409533</c:v>
+                  <c:v>2.0002800196009147</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.2340000332253496</c:v>
+                  <c:v>2.0003000225011252</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.4510818569849357</c:v>
+                  <c:v>2.0003200256013653</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.6792937038519824</c:v>
+                  <c:v>2.0003400289016375</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.9192062223138997</c:v>
+                  <c:v>2.0003600324019439</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>5.1714193186316928</c:v>
+                  <c:v>2.0003800361022863</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5.4365636569180902</c:v>
+                  <c:v>2.0004000400026669</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.7153022361263277</c:v>
+                  <c:v>2.000420044103087</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>6.0083320478928668</c:v>
+                  <c:v>2.0004400484035494</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>6.3163858193795361</c:v>
+                  <c:v>2.0004600529040557</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6.6402338454730963</c:v>
+                  <c:v>2.0004800576046082</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6.9806859149236828</c:v>
+                  <c:v>2.0005000625052087</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>7.3385933352384889</c:v>
+                  <c:v>2.000520067605859</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>7.7148510613939489</c:v>
+                  <c:v>2.0005400729065617</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>8.1103999336893509</c:v>
+                  <c:v>2.0005600784073176</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>8.5262290303376371</c:v>
+                  <c:v>2.00058008410813</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>8.963378140676129</c:v>
+                  <c:v>2.0006000900090006</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>9.4229403651814838</c:v>
+                  <c:v>2.0006200961099312</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>9.9060648487902299</c:v>
+                  <c:v>2.0006401024109235</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>10.413959654359699</c:v>
+                  <c:v>2.0006601089119802</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>10.947894783454402</c:v>
+                  <c:v>2.0006801156131027</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>11.509205352011461</c:v>
+                  <c:v>2.0007001225142931</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>12.099294928825893</c:v>
+                  <c:v>2.0007201296155532</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>12.719639045203664</c:v>
+                  <c:v>2.0007401369168858</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>13.371788884558541</c:v>
+                  <c:v>2.0007601444182925</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>14.057375161178589</c:v>
+                  <c:v>2.0007801521197748</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>14.778112197861301</c:v>
+                  <c:v>2.0008001600213356</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>15.535802212613548</c:v>
+                  <c:v>2.000820168122976</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>16.332339825135303</c:v>
+                  <c:v>2.0008401764246986</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>17.169716794355786</c:v>
+                  <c:v>2.0008601849265051</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>18.050026998868244</c:v>
+                  <c:v>2.0008801936283978</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>18.975471672717052</c:v>
+                  <c:v>2.0009002025303784</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>19.948364909629447</c:v>
+                  <c:v>2.0009202116324492</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>20.971139449455151</c:v>
+                  <c:v>2.0009402209346119</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>22.04635276128321</c:v>
+                  <c:v>2.0009602304368683</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>23.176693438446783</c:v>
+                  <c:v>2.0009802401392212</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>24.364987921406946</c:v>
+                  <c:v>2.0010002500416717</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>25.614207565326073</c:v>
+                  <c:v>2.0010202601442226</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>26.927476070003383</c:v>
+                  <c:v>2.0010402704468753</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>28.308077290751616</c:v>
+                  <c:v>2.0010602809496323</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>29.759463449745674</c:v>
+                  <c:v>2.001080291652495</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>31.285263768376343</c:v>
+                  <c:v>2.0011003025554661</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>32.88929354219411</c:v>
+                  <c:v>2.0011203136585469</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>34.575563681135279</c:v>
+                  <c:v>2.0011403249617397</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>36.348290738886135</c:v>
+                  <c:v>2.001160336465047</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>38.211907456463301</c:v>
+                  <c:v>2.0011803481684698</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>40.171073846375336</c:v>
+                  <c:v>2.0012003600720107</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>42.230688845081232</c:v>
+                  <c:v>2.0012203721756721</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>44.395902562883272</c:v>
+                  <c:v>2.0012403844794551</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>46.672129161885444</c:v>
+                  <c:v>2.001260396983362</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>49.065060394218705</c:v>
+                  <c:v>2.0012804096873955</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>51.580679834386125</c:v>
+                  <c:v>2.0013004225915565</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>54.225277841315787</c:v>
+                  <c:v>2.0013204356958476</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>57.005467287534564</c:v>
+                  <c:v>2.0013404490002711</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>59.92820009479405</c:v>
+                  <c:v>2.0013604625048287</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>63.000784617495874</c:v>
+                  <c:v>2.0013804762095218</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>66.230903917384623</c:v>
+                  <c:v>2.0014004901143534</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>69.626634975204055</c:v>
+                  <c:v>2.0014205042193249</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>73.196468887355977</c:v>
+                  <c:v>2.0014405185244386</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>76.949332098064275</c:v>
+                  <c:v>2.0014605330296962</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>80.894608720134798</c:v>
+                  <c:v>2.0014805477350999</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>85.042164000125567</c:v>
+                  <c:v>2.0015005626406515</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>89.402368986601672</c:v>
+                  <c:v>2.0015205777463532</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>93.98612646315857</c:v>
+                  <c:v>2.0015405930522068</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>98.804898211060376</c:v>
+                  <c:v>2.0015606085582149</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>103.87073366966288</c:v>
+                  <c:v>2.001580624264379</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>109.19630006628847</c:v>
+                  <c:v>2.0016006401707007</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>114.79491409089238</c:v>
+                  <c:v>2.0016206562771828</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>120.680575194724</c:v>
+                  <c:v>2.0016406725838269</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>126.86800059624669</c:v>
+                  <c:v>2.0016606890906354</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>133.37266208185031</c:v>
+                  <c:v>2.0016807057976096</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>140.21082469337571</c:v>
+                  <c:v>2.0017007227047516</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>147.39958739919157</c:v>
+                  <c:v>2.0017207398120642</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>154.9569258505218</c:v>
+                  <c:v>2.0017407571195487</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>162.90173732993628</c:v>
+                  <c:v>2.0017607746272073</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>171.25388800440118</c:v>
+                  <c:v>2.0017807923350421</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>180.03426260104362</c:v>
+                  <c:v>2.0018008102430547</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>189.26481662984813</c:v>
+                  <c:v>2.0018208283512475</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>198.96863128386772</c:v>
+                  <c:v>2.0018408466596225</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>209.16997115422845</c:v>
+                  <c:v>2.0018608651681813</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>219.89434490424705</c:v>
+                  <c:v>2.0018808838769262</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>231.16856905437533</c:v>
+                  <c:v>2.0019009027858594</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>243.02083503746994</c:v>
+                  <c:v>2.0019209218949827</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>255.48077969205784</c:v>
+                  <c:v>2.0019409412042983</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>268.57955936987105</c:v>
+                  <c:v>2.0019609607138076</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>282.34992784295372</c:v>
+                  <c:v>2.0019809804235131</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>296.8263182051532</c:v>
+                  <c:v>2.0020010003334168</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>2.0020210204435203</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>2.0020410407538263</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>2.0020610612643361</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>2.0020810819750521</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>2.0021011028859763</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>2.0021211239971106</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>2.0021411453084568</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>2.0021611668200174</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>2.0021811885317939</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>2.0022012104437885</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>2.0022212325560034</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>2.0022412548684403</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>2.0022612773811015</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>2.0022813000939887</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>2.0023013230071043</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>2.0023213461204494</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>2.0023413694340273</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>2.0023613929478388</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>2.002381416661887</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>2.0024014405761728</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>2.0024214646906988</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>2.0024414890054674</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>2.0024615135204797</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>2.0024815382357386</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>2.0025015631512453</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>2.002521588267002</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>2.002541613583011</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>2.0025616390992744</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>2.0025816648157937</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>2.0026016907325714</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>2.002621716849609</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>2.002641743166909</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>2.0026617696844733</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>2.0026817964023036</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>2.0027018233204017</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>2.0027218504387707</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>2.0027418777574115</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>2.0027619052763264</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>2.0027819329955174</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>2.002801960914987</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>2.0028219890347363</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>2.0028420173547681</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>2.0028620458750841</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>2.0028820745956866</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>2.0029021035165768</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>2.0029221326377575</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>2.00294216195923</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>2.0029621914809974</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>2.0029822212030606</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>2.0030022511254222</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>2.0030222812480836</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>2.0030423115710478</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>2.0030623420943159</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>2.0030823728178904</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>2.0031024037417726</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>2.0031224348659658</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>2.0031424661904706</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>2.00316249771529</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>2.003182529440426</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>2.0032025613658795</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>2.0032225934916537</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>2.0032426258177503</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>2.0032626583441706</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>2.0032826910709178</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>2.0033027239979928</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>2.0033227571253982</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>2.0033427904531362</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>2.0033628239812082</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>2.0033828577096164</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>2.003402891638363</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>2.0034229257674498</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>2.0034429600968791</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>2.0034629946266524</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>2.0034830293567722</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>2.0035030642872402</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>2.0035230994180586</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>2.0035431347492292</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>2.0035631702807541</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>2.0035832060126353</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>2.0036032419448753</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>2.003623278077475</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>2.0036433144104375</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>2.0036633509437638</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>2.0036833876774569</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>2.0037034246115182</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>2.0037234617459498</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>2.0037434990807537</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>2.0037635366159319</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>2.0037835743514867</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>2.0038036122874199</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>2.0038236504237332</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>2.003843688760429</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>2.0038637272975088</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>2.0038837660349755</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>2.0039038049728304</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>2.0039238441110756</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>2.0039438834497134</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>2.0039639229887451</c:v>
+                </c:pt>
+                <c:pt idx="199">
+                  <c:v>2.0039839627281739</c:v>
+                </c:pt>
+                <c:pt idx="200">
+                  <c:v>2.0040040026680006</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -952,6 +2776,7 @@
             </a:p>
           </c:txPr>
         </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1718,16 +3543,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2072,7 +3897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B3F9940-76BD-44B3-8761-831372CD6A34}">
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="37.77734375" customWidth="1"/>
@@ -2103,7 +3928,7 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0.05</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -2112,7 +3937,7 @@
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>$E$2*EXP($D$2*B3)</f>
-        <v>2.1025421927520482</v>
+        <v>2.0000200001000001</v>
       </c>
       <c r="B3">
         <f xml:space="preserve"> B2 + 1</f>
@@ -2122,7 +3947,7 @@
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" ref="A4:A67" si="0">$E$2*EXP($D$2*B4)</f>
-        <v>2.2103418361512954</v>
+        <v>2.0000400004000025</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:B67" si="1" xml:space="preserve"> B3 + 1</f>
@@ -2132,7 +3957,7 @@
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>2.3236684854565661</v>
+        <v>2.0000600009000089</v>
       </c>
       <c r="B5">
         <f t="shared" si="1"/>
@@ -2142,7 +3967,7 @@
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>2.4428055163203397</v>
+        <v>2.0000800016000215</v>
       </c>
       <c r="B6">
         <f t="shared" si="1"/>
@@ -2152,7 +3977,7 @@
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>2.5680508333754828</v>
+        <v>2.0001000025000417</v>
       </c>
       <c r="B7">
         <f t="shared" si="1"/>
@@ -2162,7 +3987,7 @@
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>2.6997176151520064</v>
+        <v>2.0001200036000721</v>
       </c>
       <c r="B8">
         <f t="shared" si="1"/>
@@ -2172,7 +3997,7 @@
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>2.8381350971865147</v>
+        <v>2.0001400049001141</v>
       </c>
       <c r="B9">
         <f t="shared" si="1"/>
@@ -2182,7 +4007,7 @@
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>2.9836493952825407</v>
+        <v>2.0001600064001708</v>
       </c>
       <c r="B10">
         <f t="shared" si="1"/>
@@ -2192,7 +4017,7 @@
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>3.1366243709803379</v>
+        <v>2.000180008100243</v>
       </c>
       <c r="B11">
         <f t="shared" si="1"/>
@@ -2202,7 +4027,7 @@
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>3.2974425414002564</v>
+        <v>2.0002000100003334</v>
       </c>
       <c r="B12">
         <f t="shared" si="1"/>
@@ -2212,7 +4037,7 @@
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>3.4665060357347905</v>
+        <v>2.0002200121004439</v>
       </c>
       <c r="B13">
         <f t="shared" si="1"/>
@@ -2222,7 +4047,7 @@
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>3.6442376007810182</v>
+        <v>2.0002400144005761</v>
       </c>
       <c r="B14">
         <f t="shared" si="1"/>
@@ -2232,7 +4057,7 @@
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>3.8310816580277924</v>
+        <v>2.0002600169007323</v>
       </c>
       <c r="B15">
         <f t="shared" si="1"/>
@@ -2242,7 +4067,7 @@
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" si="0"/>
-        <v>4.0275054149409533</v>
+        <v>2.0002800196009147</v>
       </c>
       <c r="B16">
         <f t="shared" si="1"/>
@@ -2252,7 +4077,7 @@
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="0"/>
-        <v>4.2340000332253496</v>
+        <v>2.0003000225011252</v>
       </c>
       <c r="B17">
         <f t="shared" si="1"/>
@@ -2262,7 +4087,7 @@
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="0"/>
-        <v>4.4510818569849357</v>
+        <v>2.0003200256013653</v>
       </c>
       <c r="B18">
         <f t="shared" si="1"/>
@@ -2272,7 +4097,7 @@
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" si="0"/>
-        <v>4.6792937038519824</v>
+        <v>2.0003400289016375</v>
       </c>
       <c r="B19">
         <f t="shared" si="1"/>
@@ -2282,7 +4107,7 @@
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="0"/>
-        <v>4.9192062223138997</v>
+        <v>2.0003600324019439</v>
       </c>
       <c r="B20">
         <f t="shared" si="1"/>
@@ -2292,7 +4117,7 @@
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" si="0"/>
-        <v>5.1714193186316928</v>
+        <v>2.0003800361022863</v>
       </c>
       <c r="B21">
         <f t="shared" si="1"/>
@@ -2302,7 +4127,7 @@
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22">
         <f t="shared" si="0"/>
-        <v>5.4365636569180902</v>
+        <v>2.0004000400026669</v>
       </c>
       <c r="B22">
         <f t="shared" si="1"/>
@@ -2312,7 +4137,7 @@
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" si="0"/>
-        <v>5.7153022361263277</v>
+        <v>2.000420044103087</v>
       </c>
       <c r="B23">
         <f t="shared" si="1"/>
@@ -2322,7 +4147,7 @@
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="0"/>
-        <v>6.0083320478928668</v>
+        <v>2.0004400484035494</v>
       </c>
       <c r="B24">
         <f t="shared" si="1"/>
@@ -2332,7 +4157,7 @@
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" si="0"/>
-        <v>6.3163858193795361</v>
+        <v>2.0004600529040557</v>
       </c>
       <c r="B25">
         <f t="shared" si="1"/>
@@ -2342,7 +4167,7 @@
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" si="0"/>
-        <v>6.6402338454730963</v>
+        <v>2.0004800576046082</v>
       </c>
       <c r="B26">
         <f t="shared" si="1"/>
@@ -2352,7 +4177,7 @@
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" si="0"/>
-        <v>6.9806859149236828</v>
+        <v>2.0005000625052087</v>
       </c>
       <c r="B27">
         <f t="shared" si="1"/>
@@ -2362,7 +4187,7 @@
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" si="0"/>
-        <v>7.3385933352384889</v>
+        <v>2.000520067605859</v>
       </c>
       <c r="B28">
         <f t="shared" si="1"/>
@@ -2372,7 +4197,7 @@
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" si="0"/>
-        <v>7.7148510613939489</v>
+        <v>2.0005400729065617</v>
       </c>
       <c r="B29">
         <f t="shared" si="1"/>
@@ -2382,7 +4207,7 @@
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" si="0"/>
-        <v>8.1103999336893509</v>
+        <v>2.0005600784073176</v>
       </c>
       <c r="B30">
         <f t="shared" si="1"/>
@@ -2392,7 +4217,7 @@
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
         <f t="shared" si="0"/>
-        <v>8.5262290303376371</v>
+        <v>2.00058008410813</v>
       </c>
       <c r="B31">
         <f t="shared" si="1"/>
@@ -2402,7 +4227,7 @@
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32">
         <f t="shared" si="0"/>
-        <v>8.963378140676129</v>
+        <v>2.0006000900090006</v>
       </c>
       <c r="B32">
         <f t="shared" si="1"/>
@@ -2412,7 +4237,7 @@
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
         <f t="shared" si="0"/>
-        <v>9.4229403651814838</v>
+        <v>2.0006200961099312</v>
       </c>
       <c r="B33">
         <f t="shared" si="1"/>
@@ -2422,7 +4247,7 @@
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34">
         <f t="shared" si="0"/>
-        <v>9.9060648487902299</v>
+        <v>2.0006401024109235</v>
       </c>
       <c r="B34">
         <f t="shared" si="1"/>
@@ -2432,7 +4257,7 @@
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
         <f t="shared" si="0"/>
-        <v>10.413959654359699</v>
+        <v>2.0006601089119802</v>
       </c>
       <c r="B35">
         <f t="shared" si="1"/>
@@ -2442,7 +4267,7 @@
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36">
         <f t="shared" si="0"/>
-        <v>10.947894783454402</v>
+        <v>2.0006801156131027</v>
       </c>
       <c r="B36">
         <f t="shared" si="1"/>
@@ -2452,7 +4277,7 @@
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37">
         <f t="shared" si="0"/>
-        <v>11.509205352011461</v>
+        <v>2.0007001225142931</v>
       </c>
       <c r="B37">
         <f t="shared" si="1"/>
@@ -2462,7 +4287,7 @@
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38">
         <f t="shared" si="0"/>
-        <v>12.099294928825893</v>
+        <v>2.0007201296155532</v>
       </c>
       <c r="B38">
         <f t="shared" si="1"/>
@@ -2472,7 +4297,7 @@
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39">
         <f t="shared" si="0"/>
-        <v>12.719639045203664</v>
+        <v>2.0007401369168858</v>
       </c>
       <c r="B39">
         <f t="shared" si="1"/>
@@ -2482,7 +4307,7 @@
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40">
         <f t="shared" si="0"/>
-        <v>13.371788884558541</v>
+        <v>2.0007601444182925</v>
       </c>
       <c r="B40">
         <f t="shared" si="1"/>
@@ -2492,7 +4317,7 @@
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41">
         <f t="shared" si="0"/>
-        <v>14.057375161178589</v>
+        <v>2.0007801521197748</v>
       </c>
       <c r="B41">
         <f t="shared" si="1"/>
@@ -2502,7 +4327,7 @@
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42">
         <f t="shared" si="0"/>
-        <v>14.778112197861301</v>
+        <v>2.0008001600213356</v>
       </c>
       <c r="B42">
         <f t="shared" si="1"/>
@@ -2512,7 +4337,7 @@
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43">
         <f t="shared" si="0"/>
-        <v>15.535802212613548</v>
+        <v>2.000820168122976</v>
       </c>
       <c r="B43">
         <f t="shared" si="1"/>
@@ -2522,7 +4347,7 @@
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44">
         <f t="shared" si="0"/>
-        <v>16.332339825135303</v>
+        <v>2.0008401764246986</v>
       </c>
       <c r="B44">
         <f t="shared" si="1"/>
@@ -2532,7 +4357,7 @@
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45">
         <f t="shared" si="0"/>
-        <v>17.169716794355786</v>
+        <v>2.0008601849265051</v>
       </c>
       <c r="B45">
         <f t="shared" si="1"/>
@@ -2542,7 +4367,7 @@
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46">
         <f t="shared" si="0"/>
-        <v>18.050026998868244</v>
+        <v>2.0008801936283978</v>
       </c>
       <c r="B46">
         <f t="shared" si="1"/>
@@ -2552,7 +4377,7 @@
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47">
         <f t="shared" si="0"/>
-        <v>18.975471672717052</v>
+        <v>2.0009002025303784</v>
       </c>
       <c r="B47">
         <f t="shared" si="1"/>
@@ -2562,7 +4387,7 @@
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48">
         <f t="shared" si="0"/>
-        <v>19.948364909629447</v>
+        <v>2.0009202116324492</v>
       </c>
       <c r="B48">
         <f t="shared" si="1"/>
@@ -2572,7 +4397,7 @@
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49">
         <f t="shared" si="0"/>
-        <v>20.971139449455151</v>
+        <v>2.0009402209346119</v>
       </c>
       <c r="B49">
         <f t="shared" si="1"/>
@@ -2582,7 +4407,7 @@
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50">
         <f t="shared" si="0"/>
-        <v>22.04635276128321</v>
+        <v>2.0009602304368683</v>
       </c>
       <c r="B50">
         <f t="shared" si="1"/>
@@ -2592,7 +4417,7 @@
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51">
         <f t="shared" si="0"/>
-        <v>23.176693438446783</v>
+        <v>2.0009802401392212</v>
       </c>
       <c r="B51">
         <f t="shared" si="1"/>
@@ -2602,7 +4427,7 @@
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52">
         <f t="shared" si="0"/>
-        <v>24.364987921406946</v>
+        <v>2.0010002500416717</v>
       </c>
       <c r="B52">
         <f t="shared" si="1"/>
@@ -2612,7 +4437,7 @@
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53">
         <f t="shared" si="0"/>
-        <v>25.614207565326073</v>
+        <v>2.0010202601442226</v>
       </c>
       <c r="B53">
         <f t="shared" si="1"/>
@@ -2622,7 +4447,7 @@
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54">
         <f t="shared" si="0"/>
-        <v>26.927476070003383</v>
+        <v>2.0010402704468753</v>
       </c>
       <c r="B54">
         <f t="shared" si="1"/>
@@ -2632,7 +4457,7 @@
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55">
         <f t="shared" si="0"/>
-        <v>28.308077290751616</v>
+        <v>2.0010602809496323</v>
       </c>
       <c r="B55">
         <f t="shared" si="1"/>
@@ -2642,7 +4467,7 @@
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56">
         <f t="shared" si="0"/>
-        <v>29.759463449745674</v>
+        <v>2.001080291652495</v>
       </c>
       <c r="B56">
         <f t="shared" si="1"/>
@@ -2652,7 +4477,7 @@
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57">
         <f t="shared" si="0"/>
-        <v>31.285263768376343</v>
+        <v>2.0011003025554661</v>
       </c>
       <c r="B57">
         <f t="shared" si="1"/>
@@ -2662,7 +4487,7 @@
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58">
         <f t="shared" si="0"/>
-        <v>32.88929354219411</v>
+        <v>2.0011203136585469</v>
       </c>
       <c r="B58">
         <f t="shared" si="1"/>
@@ -2672,7 +4497,7 @@
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59">
         <f t="shared" si="0"/>
-        <v>34.575563681135279</v>
+        <v>2.0011403249617397</v>
       </c>
       <c r="B59">
         <f t="shared" si="1"/>
@@ -2682,7 +4507,7 @@
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60">
         <f t="shared" si="0"/>
-        <v>36.348290738886135</v>
+        <v>2.001160336465047</v>
       </c>
       <c r="B60">
         <f t="shared" si="1"/>
@@ -2692,7 +4517,7 @@
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61">
         <f t="shared" si="0"/>
-        <v>38.211907456463301</v>
+        <v>2.0011803481684698</v>
       </c>
       <c r="B61">
         <f t="shared" si="1"/>
@@ -2702,7 +4527,7 @@
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62">
         <f t="shared" si="0"/>
-        <v>40.171073846375336</v>
+        <v>2.0012003600720107</v>
       </c>
       <c r="B62">
         <f t="shared" si="1"/>
@@ -2712,7 +4537,7 @@
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63">
         <f t="shared" si="0"/>
-        <v>42.230688845081232</v>
+        <v>2.0012203721756721</v>
       </c>
       <c r="B63">
         <f t="shared" si="1"/>
@@ -2722,7 +4547,7 @@
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64">
         <f t="shared" si="0"/>
-        <v>44.395902562883272</v>
+        <v>2.0012403844794551</v>
       </c>
       <c r="B64">
         <f t="shared" si="1"/>
@@ -2732,7 +4557,7 @@
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65">
         <f t="shared" si="0"/>
-        <v>46.672129161885444</v>
+        <v>2.001260396983362</v>
       </c>
       <c r="B65">
         <f t="shared" si="1"/>
@@ -2742,7 +4567,7 @@
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66">
         <f t="shared" si="0"/>
-        <v>49.065060394218705</v>
+        <v>2.0012804096873955</v>
       </c>
       <c r="B66">
         <f t="shared" si="1"/>
@@ -2752,7 +4577,7 @@
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67">
         <f t="shared" si="0"/>
-        <v>51.580679834386125</v>
+        <v>2.0013004225915565</v>
       </c>
       <c r="B67">
         <f t="shared" si="1"/>
@@ -2761,18 +4586,18 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68">
-        <f t="shared" ref="A68:A102" si="2">$E$2*EXP($D$2*B68)</f>
-        <v>54.225277841315787</v>
+        <f t="shared" ref="A68:A131" si="2">$E$2*EXP($D$2*B68)</f>
+        <v>2.0013204356958476</v>
       </c>
       <c r="B68">
-        <f t="shared" ref="B68:B103" si="3" xml:space="preserve"> B67 + 1</f>
+        <f t="shared" ref="B68:B131" si="3" xml:space="preserve"> B67 + 1</f>
         <v>66</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69">
         <f t="shared" si="2"/>
-        <v>57.005467287534564</v>
+        <v>2.0013404490002711</v>
       </c>
       <c r="B69">
         <f t="shared" si="3"/>
@@ -2782,7 +4607,7 @@
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70">
         <f t="shared" si="2"/>
-        <v>59.92820009479405</v>
+        <v>2.0013604625048287</v>
       </c>
       <c r="B70">
         <f t="shared" si="3"/>
@@ -2792,7 +4617,7 @@
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71">
         <f t="shared" si="2"/>
-        <v>63.000784617495874</v>
+        <v>2.0013804762095218</v>
       </c>
       <c r="B71">
         <f t="shared" si="3"/>
@@ -2802,7 +4627,7 @@
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72">
         <f t="shared" si="2"/>
-        <v>66.230903917384623</v>
+        <v>2.0014004901143534</v>
       </c>
       <c r="B72">
         <f t="shared" si="3"/>
@@ -2812,7 +4637,7 @@
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73">
         <f t="shared" si="2"/>
-        <v>69.626634975204055</v>
+        <v>2.0014205042193249</v>
       </c>
       <c r="B73">
         <f t="shared" si="3"/>
@@ -2822,7 +4647,7 @@
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74">
         <f t="shared" si="2"/>
-        <v>73.196468887355977</v>
+        <v>2.0014405185244386</v>
       </c>
       <c r="B74">
         <f t="shared" si="3"/>
@@ -2832,7 +4657,7 @@
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75">
         <f t="shared" si="2"/>
-        <v>76.949332098064275</v>
+        <v>2.0014605330296962</v>
       </c>
       <c r="B75">
         <f t="shared" si="3"/>
@@ -2842,7 +4667,7 @@
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76">
         <f t="shared" si="2"/>
-        <v>80.894608720134798</v>
+        <v>2.0014805477350999</v>
       </c>
       <c r="B76">
         <f t="shared" si="3"/>
@@ -2852,7 +4677,7 @@
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77">
         <f t="shared" si="2"/>
-        <v>85.042164000125567</v>
+        <v>2.0015005626406515</v>
       </c>
       <c r="B77">
         <f t="shared" si="3"/>
@@ -2862,7 +4687,7 @@
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78">
         <f t="shared" si="2"/>
-        <v>89.402368986601672</v>
+        <v>2.0015205777463532</v>
       </c>
       <c r="B78">
         <f t="shared" si="3"/>
@@ -2872,7 +4697,7 @@
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79">
         <f t="shared" si="2"/>
-        <v>93.98612646315857</v>
+        <v>2.0015405930522068</v>
       </c>
       <c r="B79">
         <f t="shared" si="3"/>
@@ -2882,7 +4707,7 @@
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80">
         <f t="shared" si="2"/>
-        <v>98.804898211060376</v>
+        <v>2.0015606085582149</v>
       </c>
       <c r="B80">
         <f t="shared" si="3"/>
@@ -2892,7 +4717,7 @@
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81">
         <f t="shared" si="2"/>
-        <v>103.87073366966288</v>
+        <v>2.001580624264379</v>
       </c>
       <c r="B81">
         <f t="shared" si="3"/>
@@ -2902,7 +4727,7 @@
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82">
         <f t="shared" si="2"/>
-        <v>109.19630006628847</v>
+        <v>2.0016006401707007</v>
       </c>
       <c r="B82">
         <f t="shared" si="3"/>
@@ -2912,7 +4737,7 @@
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83">
         <f t="shared" si="2"/>
-        <v>114.79491409089238</v>
+        <v>2.0016206562771828</v>
       </c>
       <c r="B83">
         <f t="shared" si="3"/>
@@ -2922,7 +4747,7 @@
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84">
         <f t="shared" si="2"/>
-        <v>120.680575194724</v>
+        <v>2.0016406725838269</v>
       </c>
       <c r="B84">
         <f t="shared" si="3"/>
@@ -2932,7 +4757,7 @@
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85">
         <f t="shared" si="2"/>
-        <v>126.86800059624669</v>
+        <v>2.0016606890906354</v>
       </c>
       <c r="B85">
         <f t="shared" si="3"/>
@@ -2942,7 +4767,7 @@
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86">
         <f t="shared" si="2"/>
-        <v>133.37266208185031</v>
+        <v>2.0016807057976096</v>
       </c>
       <c r="B86">
         <f t="shared" si="3"/>
@@ -2952,7 +4777,7 @@
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87">
         <f t="shared" si="2"/>
-        <v>140.21082469337571</v>
+        <v>2.0017007227047516</v>
       </c>
       <c r="B87">
         <f t="shared" si="3"/>
@@ -2962,7 +4787,7 @@
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88">
         <f t="shared" si="2"/>
-        <v>147.39958739919157</v>
+        <v>2.0017207398120642</v>
       </c>
       <c r="B88">
         <f t="shared" si="3"/>
@@ -2972,7 +4797,7 @@
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89">
         <f t="shared" si="2"/>
-        <v>154.9569258505218</v>
+        <v>2.0017407571195487</v>
       </c>
       <c r="B89">
         <f t="shared" si="3"/>
@@ -2982,7 +4807,7 @@
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90">
         <f t="shared" si="2"/>
-        <v>162.90173732993628</v>
+        <v>2.0017607746272073</v>
       </c>
       <c r="B90">
         <f t="shared" si="3"/>
@@ -2992,7 +4817,7 @@
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91">
         <f t="shared" si="2"/>
-        <v>171.25388800440118</v>
+        <v>2.0017807923350421</v>
       </c>
       <c r="B91">
         <f t="shared" si="3"/>
@@ -3002,7 +4827,7 @@
     <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92">
         <f t="shared" si="2"/>
-        <v>180.03426260104362</v>
+        <v>2.0018008102430547</v>
       </c>
       <c r="B92">
         <f t="shared" si="3"/>
@@ -3012,7 +4837,7 @@
     <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93">
         <f t="shared" si="2"/>
-        <v>189.26481662984813</v>
+        <v>2.0018208283512475</v>
       </c>
       <c r="B93">
         <f t="shared" si="3"/>
@@ -3022,7 +4847,7 @@
     <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94">
         <f t="shared" si="2"/>
-        <v>198.96863128386772</v>
+        <v>2.0018408466596225</v>
       </c>
       <c r="B94">
         <f t="shared" si="3"/>
@@ -3032,7 +4857,7 @@
     <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95">
         <f t="shared" si="2"/>
-        <v>209.16997115422845</v>
+        <v>2.0018608651681813</v>
       </c>
       <c r="B95">
         <f t="shared" si="3"/>
@@ -3042,7 +4867,7 @@
     <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96">
         <f t="shared" si="2"/>
-        <v>219.89434490424705</v>
+        <v>2.0018808838769262</v>
       </c>
       <c r="B96">
         <f t="shared" si="3"/>
@@ -3052,7 +4877,7 @@
     <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97">
         <f t="shared" si="2"/>
-        <v>231.16856905437533</v>
+        <v>2.0019009027858594</v>
       </c>
       <c r="B97">
         <f t="shared" si="3"/>
@@ -3062,7 +4887,7 @@
     <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98">
         <f t="shared" si="2"/>
-        <v>243.02083503746994</v>
+        <v>2.0019209218949827</v>
       </c>
       <c r="B98">
         <f t="shared" si="3"/>
@@ -3072,7 +4897,7 @@
     <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99">
         <f t="shared" si="2"/>
-        <v>255.48077969205784</v>
+        <v>2.0019409412042983</v>
       </c>
       <c r="B99">
         <f t="shared" si="3"/>
@@ -3082,7 +4907,7 @@
     <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100">
         <f t="shared" si="2"/>
-        <v>268.57955936987105</v>
+        <v>2.0019609607138076</v>
       </c>
       <c r="B100">
         <f t="shared" si="3"/>
@@ -3092,7 +4917,7 @@
     <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101">
         <f t="shared" si="2"/>
-        <v>282.34992784295372</v>
+        <v>2.0019809804235131</v>
       </c>
       <c r="B101">
         <f t="shared" si="3"/>
@@ -3102,11 +4927,1011 @@
     <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102">
         <f t="shared" si="2"/>
-        <v>296.8263182051532</v>
+        <v>2.0020010003334168</v>
       </c>
       <c r="B102">
         <f t="shared" si="3"/>
         <v>100</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103">
+        <f t="shared" si="2"/>
+        <v>2.0020210204435203</v>
+      </c>
+      <c r="B103">
+        <f t="shared" si="3"/>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104">
+        <f t="shared" si="2"/>
+        <v>2.0020410407538263</v>
+      </c>
+      <c r="B104">
+        <f t="shared" si="3"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <f t="shared" si="2"/>
+        <v>2.0020610612643361</v>
+      </c>
+      <c r="B105">
+        <f t="shared" si="3"/>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <f t="shared" si="2"/>
+        <v>2.0020810819750521</v>
+      </c>
+      <c r="B106">
+        <f t="shared" si="3"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <f t="shared" si="2"/>
+        <v>2.0021011028859763</v>
+      </c>
+      <c r="B107">
+        <f t="shared" si="3"/>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108">
+        <f t="shared" si="2"/>
+        <v>2.0021211239971106</v>
+      </c>
+      <c r="B108">
+        <f t="shared" si="3"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109">
+        <f t="shared" si="2"/>
+        <v>2.0021411453084568</v>
+      </c>
+      <c r="B109">
+        <f t="shared" si="3"/>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110">
+        <f t="shared" si="2"/>
+        <v>2.0021611668200174</v>
+      </c>
+      <c r="B110">
+        <f t="shared" si="3"/>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111">
+        <f t="shared" si="2"/>
+        <v>2.0021811885317939</v>
+      </c>
+      <c r="B111">
+        <f t="shared" si="3"/>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112">
+        <f t="shared" si="2"/>
+        <v>2.0022012104437885</v>
+      </c>
+      <c r="B112">
+        <f t="shared" si="3"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <f t="shared" si="2"/>
+        <v>2.0022212325560034</v>
+      </c>
+      <c r="B113">
+        <f t="shared" si="3"/>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <f t="shared" si="2"/>
+        <v>2.0022412548684403</v>
+      </c>
+      <c r="B114">
+        <f t="shared" si="3"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <f t="shared" si="2"/>
+        <v>2.0022612773811015</v>
+      </c>
+      <c r="B115">
+        <f t="shared" si="3"/>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <f t="shared" si="2"/>
+        <v>2.0022813000939887</v>
+      </c>
+      <c r="B116">
+        <f t="shared" si="3"/>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <f t="shared" si="2"/>
+        <v>2.0023013230071043</v>
+      </c>
+      <c r="B117">
+        <f t="shared" si="3"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <f t="shared" si="2"/>
+        <v>2.0023213461204494</v>
+      </c>
+      <c r="B118">
+        <f t="shared" si="3"/>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119">
+        <f t="shared" si="2"/>
+        <v>2.0023413694340273</v>
+      </c>
+      <c r="B119">
+        <f t="shared" si="3"/>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <f t="shared" si="2"/>
+        <v>2.0023613929478388</v>
+      </c>
+      <c r="B120">
+        <f t="shared" si="3"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <f t="shared" si="2"/>
+        <v>2.002381416661887</v>
+      </c>
+      <c r="B121">
+        <f t="shared" si="3"/>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122">
+        <f t="shared" si="2"/>
+        <v>2.0024014405761728</v>
+      </c>
+      <c r="B122">
+        <f t="shared" si="3"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123">
+        <f t="shared" si="2"/>
+        <v>2.0024214646906988</v>
+      </c>
+      <c r="B123">
+        <f t="shared" si="3"/>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124">
+        <f t="shared" si="2"/>
+        <v>2.0024414890054674</v>
+      </c>
+      <c r="B124">
+        <f t="shared" si="3"/>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125">
+        <f t="shared" si="2"/>
+        <v>2.0024615135204797</v>
+      </c>
+      <c r="B125">
+        <f t="shared" si="3"/>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126">
+        <f t="shared" si="2"/>
+        <v>2.0024815382357386</v>
+      </c>
+      <c r="B126">
+        <f t="shared" si="3"/>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127">
+        <f t="shared" si="2"/>
+        <v>2.0025015631512453</v>
+      </c>
+      <c r="B127">
+        <f t="shared" si="3"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128">
+        <f t="shared" si="2"/>
+        <v>2.002521588267002</v>
+      </c>
+      <c r="B128">
+        <f t="shared" si="3"/>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129">
+        <f t="shared" si="2"/>
+        <v>2.002541613583011</v>
+      </c>
+      <c r="B129">
+        <f t="shared" si="3"/>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130">
+        <f t="shared" si="2"/>
+        <v>2.0025616390992744</v>
+      </c>
+      <c r="B130">
+        <f t="shared" si="3"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131">
+        <f t="shared" si="2"/>
+        <v>2.0025816648157937</v>
+      </c>
+      <c r="B131">
+        <f t="shared" si="3"/>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132">
+        <f t="shared" ref="A132:A195" si="4">$E$2*EXP($D$2*B132)</f>
+        <v>2.0026016907325714</v>
+      </c>
+      <c r="B132">
+        <f t="shared" ref="B132:B195" si="5" xml:space="preserve"> B131 + 1</f>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A133">
+        <f t="shared" si="4"/>
+        <v>2.002621716849609</v>
+      </c>
+      <c r="B133">
+        <f t="shared" si="5"/>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134">
+        <f t="shared" si="4"/>
+        <v>2.002641743166909</v>
+      </c>
+      <c r="B134">
+        <f t="shared" si="5"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135">
+        <f t="shared" si="4"/>
+        <v>2.0026617696844733</v>
+      </c>
+      <c r="B135">
+        <f t="shared" si="5"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136">
+        <f t="shared" si="4"/>
+        <v>2.0026817964023036</v>
+      </c>
+      <c r="B136">
+        <f t="shared" si="5"/>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137">
+        <f t="shared" si="4"/>
+        <v>2.0027018233204017</v>
+      </c>
+      <c r="B137">
+        <f t="shared" si="5"/>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138">
+        <f t="shared" si="4"/>
+        <v>2.0027218504387707</v>
+      </c>
+      <c r="B138">
+        <f t="shared" si="5"/>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139">
+        <f t="shared" si="4"/>
+        <v>2.0027418777574115</v>
+      </c>
+      <c r="B139">
+        <f t="shared" si="5"/>
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140">
+        <f t="shared" si="4"/>
+        <v>2.0027619052763264</v>
+      </c>
+      <c r="B140">
+        <f t="shared" si="5"/>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141">
+        <f t="shared" si="4"/>
+        <v>2.0027819329955174</v>
+      </c>
+      <c r="B141">
+        <f t="shared" si="5"/>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142">
+        <f t="shared" si="4"/>
+        <v>2.002801960914987</v>
+      </c>
+      <c r="B142">
+        <f t="shared" si="5"/>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143">
+        <f t="shared" si="4"/>
+        <v>2.0028219890347363</v>
+      </c>
+      <c r="B143">
+        <f t="shared" si="5"/>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144">
+        <f t="shared" si="4"/>
+        <v>2.0028420173547681</v>
+      </c>
+      <c r="B144">
+        <f t="shared" si="5"/>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145">
+        <f t="shared" si="4"/>
+        <v>2.0028620458750841</v>
+      </c>
+      <c r="B145">
+        <f t="shared" si="5"/>
+        <v>143</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146">
+        <f t="shared" si="4"/>
+        <v>2.0028820745956866</v>
+      </c>
+      <c r="B146">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147">
+        <f t="shared" si="4"/>
+        <v>2.0029021035165768</v>
+      </c>
+      <c r="B147">
+        <f t="shared" si="5"/>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148">
+        <f t="shared" si="4"/>
+        <v>2.0029221326377575</v>
+      </c>
+      <c r="B148">
+        <f t="shared" si="5"/>
+        <v>146</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A149">
+        <f t="shared" si="4"/>
+        <v>2.00294216195923</v>
+      </c>
+      <c r="B149">
+        <f t="shared" si="5"/>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150">
+        <f t="shared" si="4"/>
+        <v>2.0029621914809974</v>
+      </c>
+      <c r="B150">
+        <f t="shared" si="5"/>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151">
+        <f t="shared" si="4"/>
+        <v>2.0029822212030606</v>
+      </c>
+      <c r="B151">
+        <f t="shared" si="5"/>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A152">
+        <f t="shared" si="4"/>
+        <v>2.0030022511254222</v>
+      </c>
+      <c r="B152">
+        <f t="shared" si="5"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153">
+        <f t="shared" si="4"/>
+        <v>2.0030222812480836</v>
+      </c>
+      <c r="B153">
+        <f t="shared" si="5"/>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154">
+        <f t="shared" si="4"/>
+        <v>2.0030423115710478</v>
+      </c>
+      <c r="B154">
+        <f t="shared" si="5"/>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155">
+        <f t="shared" si="4"/>
+        <v>2.0030623420943159</v>
+      </c>
+      <c r="B155">
+        <f t="shared" si="5"/>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156">
+        <f t="shared" si="4"/>
+        <v>2.0030823728178904</v>
+      </c>
+      <c r="B156">
+        <f t="shared" si="5"/>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A157">
+        <f t="shared" si="4"/>
+        <v>2.0031024037417726</v>
+      </c>
+      <c r="B157">
+        <f t="shared" si="5"/>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A158">
+        <f t="shared" si="4"/>
+        <v>2.0031224348659658</v>
+      </c>
+      <c r="B158">
+        <f t="shared" si="5"/>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A159">
+        <f t="shared" si="4"/>
+        <v>2.0031424661904706</v>
+      </c>
+      <c r="B159">
+        <f t="shared" si="5"/>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A160">
+        <f t="shared" si="4"/>
+        <v>2.00316249771529</v>
+      </c>
+      <c r="B160">
+        <f t="shared" si="5"/>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A161">
+        <f t="shared" si="4"/>
+        <v>2.003182529440426</v>
+      </c>
+      <c r="B161">
+        <f t="shared" si="5"/>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A162">
+        <f t="shared" si="4"/>
+        <v>2.0032025613658795</v>
+      </c>
+      <c r="B162">
+        <f t="shared" si="5"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A163">
+        <f t="shared" si="4"/>
+        <v>2.0032225934916537</v>
+      </c>
+      <c r="B163">
+        <f t="shared" si="5"/>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A164">
+        <f t="shared" si="4"/>
+        <v>2.0032426258177503</v>
+      </c>
+      <c r="B164">
+        <f t="shared" si="5"/>
+        <v>162</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A165">
+        <f t="shared" si="4"/>
+        <v>2.0032626583441706</v>
+      </c>
+      <c r="B165">
+        <f t="shared" si="5"/>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A166">
+        <f t="shared" si="4"/>
+        <v>2.0032826910709178</v>
+      </c>
+      <c r="B166">
+        <f t="shared" si="5"/>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A167">
+        <f t="shared" si="4"/>
+        <v>2.0033027239979928</v>
+      </c>
+      <c r="B167">
+        <f t="shared" si="5"/>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A168">
+        <f t="shared" si="4"/>
+        <v>2.0033227571253982</v>
+      </c>
+      <c r="B168">
+        <f t="shared" si="5"/>
+        <v>166</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A169">
+        <f t="shared" si="4"/>
+        <v>2.0033427904531362</v>
+      </c>
+      <c r="B169">
+        <f t="shared" si="5"/>
+        <v>167</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A170">
+        <f t="shared" si="4"/>
+        <v>2.0033628239812082</v>
+      </c>
+      <c r="B170">
+        <f t="shared" si="5"/>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A171">
+        <f t="shared" si="4"/>
+        <v>2.0033828577096164</v>
+      </c>
+      <c r="B171">
+        <f t="shared" si="5"/>
+        <v>169</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A172">
+        <f t="shared" si="4"/>
+        <v>2.003402891638363</v>
+      </c>
+      <c r="B172">
+        <f t="shared" si="5"/>
+        <v>170</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A173">
+        <f t="shared" si="4"/>
+        <v>2.0034229257674498</v>
+      </c>
+      <c r="B173">
+        <f t="shared" si="5"/>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A174">
+        <f t="shared" si="4"/>
+        <v>2.0034429600968791</v>
+      </c>
+      <c r="B174">
+        <f t="shared" si="5"/>
+        <v>172</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A175">
+        <f t="shared" si="4"/>
+        <v>2.0034629946266524</v>
+      </c>
+      <c r="B175">
+        <f t="shared" si="5"/>
+        <v>173</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A176">
+        <f t="shared" si="4"/>
+        <v>2.0034830293567722</v>
+      </c>
+      <c r="B176">
+        <f t="shared" si="5"/>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A177">
+        <f t="shared" si="4"/>
+        <v>2.0035030642872402</v>
+      </c>
+      <c r="B177">
+        <f t="shared" si="5"/>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A178">
+        <f t="shared" si="4"/>
+        <v>2.0035230994180586</v>
+      </c>
+      <c r="B178">
+        <f t="shared" si="5"/>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A179">
+        <f t="shared" si="4"/>
+        <v>2.0035431347492292</v>
+      </c>
+      <c r="B179">
+        <f t="shared" si="5"/>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A180">
+        <f t="shared" si="4"/>
+        <v>2.0035631702807541</v>
+      </c>
+      <c r="B180">
+        <f t="shared" si="5"/>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A181">
+        <f t="shared" si="4"/>
+        <v>2.0035832060126353</v>
+      </c>
+      <c r="B181">
+        <f t="shared" si="5"/>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A182">
+        <f t="shared" si="4"/>
+        <v>2.0036032419448753</v>
+      </c>
+      <c r="B182">
+        <f t="shared" si="5"/>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A183">
+        <f t="shared" si="4"/>
+        <v>2.003623278077475</v>
+      </c>
+      <c r="B183">
+        <f t="shared" si="5"/>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A184">
+        <f t="shared" si="4"/>
+        <v>2.0036433144104375</v>
+      </c>
+      <c r="B184">
+        <f t="shared" si="5"/>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A185">
+        <f t="shared" si="4"/>
+        <v>2.0036633509437638</v>
+      </c>
+      <c r="B185">
+        <f t="shared" si="5"/>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A186">
+        <f t="shared" si="4"/>
+        <v>2.0036833876774569</v>
+      </c>
+      <c r="B186">
+        <f t="shared" si="5"/>
+        <v>184</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A187">
+        <f t="shared" si="4"/>
+        <v>2.0037034246115182</v>
+      </c>
+      <c r="B187">
+        <f t="shared" si="5"/>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A188">
+        <f t="shared" si="4"/>
+        <v>2.0037234617459498</v>
+      </c>
+      <c r="B188">
+        <f t="shared" si="5"/>
+        <v>186</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A189">
+        <f t="shared" si="4"/>
+        <v>2.0037434990807537</v>
+      </c>
+      <c r="B189">
+        <f t="shared" si="5"/>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A190">
+        <f t="shared" si="4"/>
+        <v>2.0037635366159319</v>
+      </c>
+      <c r="B190">
+        <f t="shared" si="5"/>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A191">
+        <f t="shared" si="4"/>
+        <v>2.0037835743514867</v>
+      </c>
+      <c r="B191">
+        <f t="shared" si="5"/>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A192">
+        <f t="shared" si="4"/>
+        <v>2.0038036122874199</v>
+      </c>
+      <c r="B192">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A193">
+        <f t="shared" si="4"/>
+        <v>2.0038236504237332</v>
+      </c>
+      <c r="B193">
+        <f t="shared" si="5"/>
+        <v>191</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A194">
+        <f t="shared" si="4"/>
+        <v>2.003843688760429</v>
+      </c>
+      <c r="B194">
+        <f t="shared" si="5"/>
+        <v>192</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A195">
+        <f t="shared" si="4"/>
+        <v>2.0038637272975088</v>
+      </c>
+      <c r="B195">
+        <f t="shared" si="5"/>
+        <v>193</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A196">
+        <f t="shared" ref="A196:A202" si="6">$E$2*EXP($D$2*B196)</f>
+        <v>2.0038837660349755</v>
+      </c>
+      <c r="B196">
+        <f t="shared" ref="B196:B220" si="7" xml:space="preserve"> B195 + 1</f>
+        <v>194</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A197">
+        <f t="shared" si="6"/>
+        <v>2.0039038049728304</v>
+      </c>
+      <c r="B197">
+        <f t="shared" si="7"/>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A198">
+        <f t="shared" si="6"/>
+        <v>2.0039238441110756</v>
+      </c>
+      <c r="B198">
+        <f t="shared" si="7"/>
+        <v>196</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A199">
+        <f t="shared" si="6"/>
+        <v>2.0039438834497134</v>
+      </c>
+      <c r="B199">
+        <f t="shared" si="7"/>
+        <v>197</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A200">
+        <f t="shared" si="6"/>
+        <v>2.0039639229887451</v>
+      </c>
+      <c r="B200">
+        <f t="shared" si="7"/>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A201">
+        <f t="shared" si="6"/>
+        <v>2.0039839627281739</v>
+      </c>
+      <c r="B201">
+        <f t="shared" si="7"/>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A202">
+        <f t="shared" si="6"/>
+        <v>2.0040040026680006</v>
+      </c>
+      <c r="B202">
+        <f t="shared" si="7"/>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>